<commit_message>
Changement dans les dates, amélioration de de la charte graphique
</commit_message>
<xml_diff>
--- a/Documentation/Dates projet FISCHER-NOTAR.xlsx
+++ b/Documentation/Dates projet FISCHER-NOTAR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eleve\Desktop\Cours\BTS\1ère année\U5.6 - AP1 - P. Schlegel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ylian\Desktop\Cours\BTS\1ère année\U5 - AP1 - P. Schlegel\Projet\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C038C3C4-A932-41AA-AD74-0307D283EDCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF23C9F3-39A8-473B-B9EB-CF9522EEE719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{05ADEA78-6E4E-4141-8E80-F03980EA277B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{05ADEA78-6E4E-4141-8E80-F03980EA277B}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="36">
   <si>
     <t>Semaine 36</t>
   </si>
@@ -144,6 +144,9 @@
   </si>
   <si>
     <t>préparation soutenance</t>
+  </si>
+  <si>
+    <t>HTML</t>
   </si>
 </sst>
 </file>
@@ -525,9 +528,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{242BAF26-C150-4EF6-9608-75DE8CEA658B}">
   <dimension ref="A1:C23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -536,7 +539,7 @@
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -545,7 +548,7 @@
       </c>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -554,7 +557,7 @@
       </c>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -563,7 +566,7 @@
       </c>
       <c r="C4" s="1"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -572,7 +575,7 @@
       </c>
       <c r="C5" s="1"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -581,7 +584,7 @@
       </c>
       <c r="C6" s="1"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -590,7 +593,7 @@
       </c>
       <c r="C7" s="1"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -599,7 +602,7 @@
       </c>
       <c r="C8" s="1"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -608,16 +611,16 @@
       </c>
       <c r="C9" s="1"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C10" s="1"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -626,7 +629,7 @@
       </c>
       <c r="C11" s="1"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -635,7 +638,7 @@
       </c>
       <c r="C12" s="1"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -644,7 +647,7 @@
       </c>
       <c r="C13" s="1"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -653,7 +656,7 @@
       </c>
       <c r="C14" s="1"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -662,7 +665,7 @@
       </c>
       <c r="C15" s="1"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -671,7 +674,7 @@
       </c>
       <c r="C16" s="1"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -680,7 +683,7 @@
       </c>
       <c r="C17" s="1"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -689,7 +692,7 @@
       </c>
       <c r="C18" s="1"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -698,7 +701,7 @@
       </c>
       <c r="C19" s="1"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -707,7 +710,7 @@
       </c>
       <c r="C20" s="1"/>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -716,7 +719,7 @@
       </c>
       <c r="C21" s="1"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -725,7 +728,7 @@
       </c>
       <c r="C22" s="1"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -736,11 +739,12 @@
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
@@ -753,12 +757,11 @@
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>